<commit_message>
update html et script
</commit_message>
<xml_diff>
--- a/tables_clusters_par_block/tableau_recapitulatif_clustvar_final.xlsx
+++ b/tables_clusters_par_block/tableau_recapitulatif_clustvar_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\g.martet\Documents\functional_study\tables_clusters_par_block\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF6721F4-DDC4-43D0-939A-4FF2C58C7F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE0F8479-FA79-45EA-9187-4FB4D71A9E0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -738,20 +738,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L87"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -777,7 +777,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -801,7 +801,7 @@
       </c>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
@@ -827,7 +827,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
@@ -851,7 +851,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -875,7 +875,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -895,7 +895,7 @@
       </c>
       <c r="H6" s="1"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>17</v>
       </c>
@@ -917,7 +917,7 @@
       </c>
       <c r="H7" s="1"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -945,7 +945,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -969,7 +969,7 @@
       </c>
       <c r="H9" s="1"/>
     </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -995,7 +995,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
@@ -1067,7 +1067,7 @@
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
     </row>
-    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="H15" s="1"/>
     </row>
-    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -1135,7 +1135,7 @@
       </c>
       <c r="H16" s="1"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
@@ -1161,7 +1161,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="H18" s="1"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -1211,7 +1211,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>17</v>
       </c>
@@ -1233,7 +1233,7 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
     </row>
-    <row r="21" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="1" t="s">
         <v>17</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>17</v>
       </c>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="H23" s="1"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>17</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>17</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>17</v>
       </c>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="H26" s="1"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>17</v>
       </c>
@@ -1393,7 +1393,7 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>17</v>
       </c>
@@ -1409,7 +1409,7 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>
-    <row r="29" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="2" t="s">
         <v>17</v>
       </c>
@@ -1423,7 +1423,7 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="3" t="s">
         <v>8</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>9</v>
       </c>
       <c r="C30" s="3"/>
-      <c r="D30" s="4" t="s">
+      <c r="D30" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -1441,7 +1441,7 @@
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
     </row>
-    <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="1" t="s">
         <v>8</v>
       </c>
@@ -1457,7 +1457,7 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
     </row>
-    <row r="32" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="1" t="s">
         <v>8</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="1" t="s">
         <v>8</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="1" t="s">
         <v>8</v>
       </c>
@@ -1523,7 +1523,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="1" t="s">
         <v>8</v>
       </c>
@@ -1541,7 +1541,7 @@
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
     </row>
-    <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>8</v>
       </c>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="H36" s="1"/>
     </row>
-    <row r="37" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="1" t="s">
         <v>8</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>8</v>
       </c>
@@ -1605,7 +1605,7 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>8</v>
       </c>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="H39" s="1"/>
     </row>
-    <row r="40" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>8</v>
       </c>
@@ -1637,7 +1637,7 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
     </row>
-    <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="1" t="s">
         <v>8</v>
       </c>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="H41" s="1"/>
     </row>
-    <row r="42" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="1" t="s">
         <v>8</v>
       </c>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="H42" s="1"/>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>8</v>
       </c>
@@ -1703,7 +1703,7 @@
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>8</v>
       </c>
@@ -1717,7 +1717,7 @@
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>8</v>
       </c>
@@ -1735,7 +1735,7 @@
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>8</v>
       </c>
@@ -1757,7 +1757,7 @@
       </c>
       <c r="H46" s="1"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>8</v>
       </c>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="H47" s="1"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>8</v>
       </c>
@@ -1793,7 +1793,7 @@
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
     </row>
-    <row r="49" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="1" t="s">
         <v>8</v>
       </c>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="H49" s="1"/>
     </row>
-    <row r="50" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="1" t="s">
         <v>8</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>8</v>
       </c>
@@ -1851,7 +1851,7 @@
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>8</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="1" t="s">
         <v>8</v>
       </c>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="H53" s="1"/>
     </row>
-    <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="1" t="s">
         <v>8</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>8</v>
       </c>
@@ -1937,7 +1937,7 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>8</v>
       </c>
@@ -1955,7 +1955,7 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>8</v>
       </c>
@@ -1969,7 +1969,7 @@
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>77</v>
       </c>
@@ -1995,7 +1995,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>77</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="1" t="s">
         <v>77</v>
       </c>
@@ -2047,7 +2047,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="1" t="s">
         <v>77</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>77</v>
       </c>
@@ -2087,7 +2087,7 @@
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>77</v>
       </c>
@@ -2103,7 +2103,7 @@
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
     </row>
-    <row r="64" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="1" t="s">
         <v>77</v>
       </c>
@@ -2117,7 +2117,7 @@
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
     </row>
-    <row r="65" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="1" t="s">
         <v>77</v>
       </c>
@@ -2143,7 +2143,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>77</v>
       </c>
@@ -2159,7 +2159,7 @@
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>77</v>
       </c>
@@ -2175,7 +2175,7 @@
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
     </row>
-    <row r="68" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="2" t="s">
         <v>77</v>
       </c>
@@ -2189,7 +2189,7 @@
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="3" t="s">
         <v>43</v>
       </c>
@@ -2207,7 +2207,7 @@
       <c r="G69" s="3"/>
       <c r="H69" s="3"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>43</v>
       </c>
@@ -2227,7 +2227,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>43</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>43</v>
       </c>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="H72" s="1"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>43</v>
       </c>
@@ -2291,7 +2291,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="1" t="s">
         <v>43</v>
       </c>
@@ -2305,7 +2305,7 @@
       <c r="G74" s="1"/>
       <c r="H74" s="1"/>
     </row>
-    <row r="75" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="1" t="s">
         <v>43</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>43</v>
       </c>
@@ -2347,7 +2347,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>43</v>
       </c>
@@ -2361,7 +2361,7 @@
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
     </row>
-    <row r="78" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="1" t="s">
         <v>43</v>
       </c>
@@ -2385,7 +2385,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="1" t="s">
         <v>43</v>
       </c>
@@ -2411,7 +2411,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>43</v>
       </c>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="H80" s="1"/>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>43</v>
       </c>
@@ -2445,7 +2445,7 @@
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>43</v>
       </c>
@@ -2463,7 +2463,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>43</v>
       </c>
@@ -2487,7 +2487,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>43</v>
       </c>
@@ -2505,7 +2505,7 @@
       <c r="G84" s="1"/>
       <c r="H84" s="1"/>
     </row>
-    <row r="85" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="1" t="s">
         <v>43</v>
       </c>
@@ -2525,7 +2525,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="1" t="s">
         <v>43</v>
       </c>
@@ -2545,7 +2545,7 @@
       <c r="G86" s="1"/>
       <c r="H86" s="1"/>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>43</v>
       </c>

</xml_diff>